<commit_message>
Test: add dummy event to PE calendar
</commit_message>
<xml_diff>
--- a/data/pe_event_calendar_2026.xlsx
+++ b/data/pe_event_calendar_2026.xlsx
@@ -2928,37 +2928,37 @@
     <row r="53" ht="28" customHeight="1">
       <c r="A53" s="13" t="inlineStr">
         <is>
-          <t>September 2026 (tbd)</t>
+          <t>20.03.2026</t>
         </is>
       </c>
       <c r="B53" s="13" t="inlineStr">
         <is>
-          <t>IPEM Paris 2026</t>
+          <t>TEST EVENT — Bitte ignorieren</t>
         </is>
       </c>
       <c r="C53" s="14" t="inlineStr">
         <is>
-          <t>IPEM</t>
+          <t>HAC Test</t>
         </is>
       </c>
       <c r="D53" s="14" t="inlineStr">
         <is>
-          <t>Paris</t>
+          <t>München</t>
         </is>
       </c>
       <c r="E53" s="15" t="inlineStr">
         <is>
-          <t>FR</t>
+          <t>DE</t>
         </is>
       </c>
       <c r="F53" s="16" t="inlineStr">
         <is>
-          <t>tbc</t>
+          <t>Free</t>
         </is>
       </c>
       <c r="G53" s="17" t="inlineStr">
         <is>
-          <t>https://www.ipem-market.com/</t>
+          <t>https://example.com</t>
         </is>
       </c>
       <c r="H53" s="16" t="inlineStr">
@@ -2968,7 +2968,7 @@
       </c>
       <c r="I53" s="16" t="inlineStr">
         <is>
-          <t>Conference</t>
+          <t>Test</t>
         </is>
       </c>
     </row>
@@ -3118,225 +3118,4 @@
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
-</file>
-
-<file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Dokument" ma:contentTypeID="0x010100D64F4D755BE2E349AF8B57C761DE3BFA" ma:contentTypeVersion="10" ma:contentTypeDescription="Ein neues Dokument erstellen." ma:contentTypeScope="" ma:versionID="7c372a3e51f366a63ca64bb29072728e">
-  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="b541a2e5-6919-4c18-819d-6f9beb94c080" xmlns:ns3="239df7f2-98c0-4b21-bce8-bfddaf72a22d" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="40f1e2ce5c9d8c089f89cb07a6218374" ns2:_="" ns3:_="">
-    <xsd:import namespace="b541a2e5-6919-4c18-819d-6f9beb94c080"/>
-    <xsd:import namespace="239df7f2-98c0-4b21-bce8-bfddaf72a22d"/>
-    <xsd:element name="properties">
-      <xsd:complexType>
-        <xsd:sequence>
-          <xsd:element name="documentManagement">
-            <xsd:complexType>
-              <xsd:all>
-                <xsd:element ref="ns2:MediaServiceMetadata" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceFastMetadata" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceSearchProperties" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceDateTaken" minOccurs="0"/>
-                <xsd:element ref="ns2:lcf76f155ced4ddcb4097134ff3c332f" minOccurs="0"/>
-                <xsd:element ref="ns3:TaxCatchAll" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceOCR" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceGenerationTime" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceEventHashCode" minOccurs="0"/>
-              </xsd:all>
-            </xsd:complexType>
-          </xsd:element>
-        </xsd:sequence>
-      </xsd:complexType>
-    </xsd:element>
-  </xsd:schema>
-  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="b541a2e5-6919-4c18-819d-6f9beb94c080" elementFormDefault="qualified">
-    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <xsd:element name="MediaServiceMetadata" ma:index="8" nillable="true" ma:displayName="MediaServiceMetadata" ma:hidden="true" ma:internalName="MediaServiceMetadata" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Note"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceFastMetadata" ma:index="9" nillable="true" ma:displayName="MediaServiceFastMetadata" ma:hidden="true" ma:internalName="MediaServiceFastMetadata" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Note"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceSearchProperties" ma:index="10" nillable="true" ma:displayName="MediaServiceSearchProperties" ma:hidden="true" ma:internalName="MediaServiceSearchProperties" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Note"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceDateTaken" ma:index="11" nillable="true" ma:displayName="MediaServiceDateTaken" ma:hidden="true" ma:indexed="true" ma:internalName="MediaServiceDateTaken" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Text"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="lcf76f155ced4ddcb4097134ff3c332f" ma:index="13" nillable="true" ma:taxonomy="true" ma:internalName="lcf76f155ced4ddcb4097134ff3c332f" ma:taxonomyFieldName="MediaServiceImageTags" ma:displayName="Bildmarkierungen" ma:readOnly="false" ma:fieldId="{5cf76f15-5ced-4ddc-b409-7134ff3c332f}" ma:taxonomyMulti="true" ma:sspId="346b11dc-3bcc-47ab-87c3-03d1ecdedb00" ma:termSetId="09814cd3-568e-fe90-9814-8d621ff8fb84" ma:anchorId="fba54fb3-c3e1-fe81-a776-ca4b69148c4d" ma:open="true" ma:isKeyword="false">
-      <xsd:complexType>
-        <xsd:sequence>
-          <xsd:element ref="pc:Terms" minOccurs="0" maxOccurs="1"/>
-        </xsd:sequence>
-      </xsd:complexType>
-    </xsd:element>
-    <xsd:element name="MediaServiceOCR" ma:index="15" nillable="true" ma:displayName="Extracted Text" ma:internalName="MediaServiceOCR" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Note">
-          <xsd:maxLength value="255"/>
-        </xsd:restriction>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceGenerationTime" ma:index="16" nillable="true" ma:displayName="MediaServiceGenerationTime" ma:hidden="true" ma:internalName="MediaServiceGenerationTime" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Text"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceEventHashCode" ma:index="17" nillable="true" ma:displayName="MediaServiceEventHashCode" ma:hidden="true" ma:internalName="MediaServiceEventHashCode" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Text"/>
-      </xsd:simpleType>
-    </xsd:element>
-  </xsd:schema>
-  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="239df7f2-98c0-4b21-bce8-bfddaf72a22d" elementFormDefault="qualified">
-    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <xsd:element name="TaxCatchAll" ma:index="14" nillable="true" ma:displayName="Taxonomy Catch All Column" ma:hidden="true" ma:list="{7a7057d5-3953-4235-9769-b5806729f79f}" ma:internalName="TaxCatchAll" ma:showField="CatchAllData" ma:web="239df7f2-98c0-4b21-bce8-bfddaf72a22d">
-      <xsd:complexType>
-        <xsd:complexContent>
-          <xsd:extension base="dms:MultiChoiceLookup">
-            <xsd:sequence>
-              <xsd:element name="Value" type="dms:Lookup" maxOccurs="unbounded" minOccurs="0" nillable="true"/>
-            </xsd:sequence>
-          </xsd:extension>
-        </xsd:complexContent>
-      </xsd:complexType>
-    </xsd:element>
-  </xsd:schema>
-  <xsd:schema xmlns="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:dc="http://purl.org/dc/elements/1.1/" xmlns:dcterms="http://purl.org/dc/terms/" xmlns:odoc="http://schemas.microsoft.com/internal/obd" targetNamespace="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" elementFormDefault="qualified" attributeFormDefault="unqualified" blockDefault="#all">
-    <xsd:import namespace="http://purl.org/dc/elements/1.1/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dc.xsd"/>
-    <xsd:import namespace="http://purl.org/dc/terms/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dcterms.xsd"/>
-    <xsd:element name="coreProperties" type="CT_coreProperties"/>
-    <xsd:complexType name="CT_coreProperties">
-      <xsd:all>
-        <xsd:element ref="dc:creator" minOccurs="0" maxOccurs="1"/>
-        <xsd:element ref="dcterms:created" minOccurs="0" maxOccurs="1"/>
-        <xsd:element ref="dc:identifier" minOccurs="0" maxOccurs="1"/>
-        <xsd:element name="contentType" minOccurs="0" maxOccurs="1" type="xsd:string" ma:index="0" ma:displayName="Inhaltstyp"/>
-        <xsd:element ref="dc:title" minOccurs="0" maxOccurs="1" ma:index="4" ma:displayName="Titel"/>
-        <xsd:element ref="dc:subject" minOccurs="0" maxOccurs="1"/>
-        <xsd:element ref="dc:description" minOccurs="0" maxOccurs="1"/>
-        <xsd:element name="keywords" minOccurs="0" maxOccurs="1" type="xsd:string"/>
-        <xsd:element ref="dc:language" minOccurs="0" maxOccurs="1"/>
-        <xsd:element name="category" minOccurs="0" maxOccurs="1" type="xsd:string"/>
-        <xsd:element name="version" minOccurs="0" maxOccurs="1" type="xsd:string"/>
-        <xsd:element name="revision" minOccurs="0" maxOccurs="1" type="xsd:string">
-          <xsd:annotation>
-            <xsd:documentation>
-                        This value indicates the number of saves or revisions. The application is responsible for updating this value after each revision.
-                    </xsd:documentation>
-          </xsd:annotation>
-        </xsd:element>
-        <xsd:element name="lastModifiedBy" minOccurs="0" maxOccurs="1" type="xsd:string"/>
-        <xsd:element ref="dcterms:modified" minOccurs="0" maxOccurs="1"/>
-        <xsd:element name="contentStatus" minOccurs="0" maxOccurs="1" type="xsd:string"/>
-      </xsd:all>
-    </xsd:complexType>
-  </xsd:schema>
-  <xs:schema xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" xmlns:xs="http://www.w3.org/2001/XMLSchema" targetNamespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" elementFormDefault="qualified" attributeFormDefault="unqualified">
-    <xs:element name="Person">
-      <xs:complexType>
-        <xs:sequence>
-          <xs:element ref="pc:DisplayName" minOccurs="0"/>
-          <xs:element ref="pc:AccountId" minOccurs="0"/>
-          <xs:element ref="pc:AccountType" minOccurs="0"/>
-        </xs:sequence>
-      </xs:complexType>
-    </xs:element>
-    <xs:element name="DisplayName" type="xs:string"/>
-    <xs:element name="AccountId" type="xs:string"/>
-    <xs:element name="AccountType" type="xs:string"/>
-    <xs:element name="BDCAssociatedEntity">
-      <xs:complexType>
-        <xs:sequence>
-          <xs:element ref="pc:BDCEntity" minOccurs="0" maxOccurs="unbounded"/>
-        </xs:sequence>
-        <xs:attribute ref="pc:EntityNamespace"/>
-        <xs:attribute ref="pc:EntityName"/>
-        <xs:attribute ref="pc:SystemInstanceName"/>
-        <xs:attribute ref="pc:AssociationName"/>
-      </xs:complexType>
-    </xs:element>
-    <xs:attribute name="EntityNamespace" type="xs:string"/>
-    <xs:attribute name="EntityName" type="xs:string"/>
-    <xs:attribute name="SystemInstanceName" type="xs:string"/>
-    <xs:attribute name="AssociationName" type="xs:string"/>
-    <xs:element name="BDCEntity">
-      <xs:complexType>
-        <xs:sequence>
-          <xs:element ref="pc:EntityDisplayName" minOccurs="0"/>
-          <xs:element ref="pc:EntityInstanceReference" minOccurs="0"/>
-          <xs:element ref="pc:EntityId1" minOccurs="0"/>
-          <xs:element ref="pc:EntityId2" minOccurs="0"/>
-          <xs:element ref="pc:EntityId3" minOccurs="0"/>
-          <xs:element ref="pc:EntityId4" minOccurs="0"/>
-          <xs:element ref="pc:EntityId5" minOccurs="0"/>
-        </xs:sequence>
-      </xs:complexType>
-    </xs:element>
-    <xs:element name="EntityDisplayName" type="xs:string"/>
-    <xs:element name="EntityInstanceReference" type="xs:string"/>
-    <xs:element name="EntityId1" type="xs:string"/>
-    <xs:element name="EntityId2" type="xs:string"/>
-    <xs:element name="EntityId3" type="xs:string"/>
-    <xs:element name="EntityId4" type="xs:string"/>
-    <xs:element name="EntityId5" type="xs:string"/>
-    <xs:element name="Terms">
-      <xs:complexType>
-        <xs:sequence>
-          <xs:element ref="pc:TermInfo" minOccurs="0" maxOccurs="unbounded"/>
-        </xs:sequence>
-      </xs:complexType>
-    </xs:element>
-    <xs:element name="TermInfo">
-      <xs:complexType>
-        <xs:sequence>
-          <xs:element ref="pc:TermName" minOccurs="0"/>
-          <xs:element ref="pc:TermId" minOccurs="0"/>
-        </xs:sequence>
-      </xs:complexType>
-    </xs:element>
-    <xs:element name="TermName" type="xs:string"/>
-    <xs:element name="TermId" type="xs:string"/>
-  </xs:schema>
-</ct:contentTypeSchema>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <TaxCatchAll xmlns="239df7f2-98c0-4b21-bce8-bfddaf72a22d" xsi:nil="true"/>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="b541a2e5-6919-4c18-819d-6f9beb94c080">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{85ABDEEF-B746-4A18-A0B8-B52BDFB93D94}"/>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{730545D2-A3D7-414D-89D1-23800440E25F}"/>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{CF282199-C3C6-4893-8DA5-D9F1512CDF1B}"/>
 </file>
</xml_diff>

<commit_message>
Clean up: remove all test events from Excel
</commit_message>
<xml_diff>
--- a/data/pe_event_calendar_2026.xlsx
+++ b/data/pe_event_calendar_2026.xlsx
@@ -641,7 +641,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S54"/>
+  <dimension ref="A1:S52"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" style="37" min="1" max="1"/>
@@ -3042,98 +3042,7 @@
         </is>
       </c>
     </row>
-    <row r="53" ht="28" customHeight="1" s="37">
-      <c r="A53" s="11" t="inlineStr">
-        <is>
-          <t>20.03.2026</t>
-        </is>
-      </c>
-      <c r="B53" s="11" t="inlineStr">
-        <is>
-          <t>TEST EVENT — Bitte ignorieren</t>
-        </is>
-      </c>
-      <c r="C53" s="12" t="inlineStr">
-        <is>
-          <t>HAC Test</t>
-        </is>
-      </c>
-      <c r="D53" s="12" t="inlineStr">
-        <is>
-          <t>München</t>
-        </is>
-      </c>
-      <c r="E53" s="13" t="inlineStr">
-        <is>
-          <t>DE</t>
-        </is>
-      </c>
-      <c r="F53" s="14" t="inlineStr">
-        <is>
-          <t>Free</t>
-        </is>
-      </c>
-      <c r="G53" s="15" t="inlineStr">
-        <is>
-          <t>https://example.com</t>
-        </is>
-      </c>
-      <c r="H53" s="14" t="inlineStr">
-        <is>
-          <t>Upcoming</t>
-        </is>
-      </c>
-      <c r="I53" s="14" t="inlineStr">
-        <is>
-          <t>Test</t>
-        </is>
-      </c>
-    </row>
-    <row r="54">
-      <c r="A54" s="40" t="n">
-        <v>46330</v>
-      </c>
-      <c r="B54" s="41" t="inlineStr">
-        <is>
-          <t>TEST 123123</t>
-        </is>
-      </c>
-      <c r="C54" s="42" t="inlineStr">
-        <is>
-          <t>CF TEST</t>
-        </is>
-      </c>
-      <c r="D54" s="42" t="inlineStr">
-        <is>
-          <t>Düsseldorf</t>
-        </is>
-      </c>
-      <c r="E54" s="43" t="inlineStr">
-        <is>
-          <t>UK</t>
-        </is>
-      </c>
-      <c r="F54" s="44" t="inlineStr">
-        <is>
-          <t>Free</t>
-        </is>
-      </c>
-      <c r="G54" s="45" t="inlineStr">
-        <is>
-          <t>https://www.tactus.works</t>
-        </is>
-      </c>
-      <c r="H54" s="44" t="inlineStr">
-        <is>
-          <t>Upcoming</t>
-        </is>
-      </c>
-      <c r="I54" s="44" t="inlineStr">
-        <is>
-          <t>Test</t>
-        </is>
-      </c>
-    </row>
+    <row r="53" ht="28" customHeight="1" s="37"/>
   </sheetData>
   <autoFilter ref="A4:I53"/>
   <mergeCells count="3">
@@ -3190,8 +3099,6 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G50" r:id="rId46"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G51" r:id="rId47"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G52" r:id="rId48"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G53" r:id="rId49"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G54" r:id="rId50"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>